<commit_message>
ajustes ranking seleccion de var en exploracion
</commit_message>
<xml_diff>
--- a/data/plantilla_exploracion_modelo.xlsx
+++ b/data/plantilla_exploracion_modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\gdrive_luisflorez\Mi unidad\PROYECTOS_LF\ProyectosE2\LBEn_EDIF_app\LBEn_APP_Resol016\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D9F095-F833-4FC3-B19B-81FDE9000AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5020FC6F-3CC0-4C0D-B147-0F0A2D743397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
   <si>
     <t>SISTEMA DE GESTIÓN LBEn — EXPLORACIÓN Y SELECCIÓN DE MODELO</t>
   </si>
@@ -247,12 +247,14 @@
     <t>No se incluye. La correlación no distingue del azar.</t>
   </si>
   <si>
+    <t>Período Análisis:</t>
+  </si>
+  <si>
+    <t>Sugerencia</t>
+  </si>
+  <si>
     <t>← Esta sección es completada automáticamente por la APP al ejecutar el análisis de exploración.
-Los valores de r, p-valor y la decisión de significancia se actualizan con los datos de [Periodo_Análisis].
-La fila 'Ejemplo_Var3' es ilustrativa y será reemplazada por las variables reales del proyecto.</t>
-  </si>
-  <si>
-    <t>Período Análisis:</t>
+Los valores de r, p-valor y la decisión de significancia se actualizan con los datos de [Periodo_Análisis].</t>
   </si>
 </sst>
 </file>
@@ -425,7 +427,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -448,11 +450,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -550,6 +561,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -950,7 +964,7 @@
     </row>
     <row r="13" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="19"/>
@@ -1088,7 +1102,7 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
-    <col min="8" max="8" width="3" customWidth="1"/>
+    <col min="8" max="8" width="30.54296875" customWidth="1"/>
     <col min="11" max="11" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.6328125" bestFit="1" customWidth="1"/>
@@ -1256,14 +1270,15 @@
       <c r="P8" s="19"/>
     </row>
     <row r="9" spans="2:16" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
     </row>
     <row r="10" spans="2:16" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="10" t="s">
@@ -1284,8 +1299,11 @@
       <c r="G10" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="H10" s="10" t="s">
+        <v>72</v>
+      </c>
       <c r="K10" s="27" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L10" s="19"/>
       <c r="M10" s="19"/>
@@ -1310,6 +1328,9 @@
         <v>43</v>
       </c>
       <c r="G11" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1343,7 +1364,7 @@
     <mergeCell ref="O6:P6"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B9:H9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>